<commit_message>
Add barangay CapBuild and action plan target fields
</commit_message>
<xml_diff>
--- a/implementation-status/helpers/Program_Targets_Template.xlsx
+++ b/implementation-status/helpers/Program_Targets_Template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="17">
   <si>
     <t>PROVINCE</t>
   </si>
@@ -39,6 +39,12 @@
   </si>
   <si>
     <t>BINHI TARGET</t>
+  </si>
+  <si>
+    <t>CAPBUILD TARGET</t>
+  </si>
+  <si>
+    <t>COMMUNITY ACTION PLAN TARGET</t>
   </si>
   <si>
     <t>TARGET PARTNER-BENEFICIARIES</t>
@@ -399,7 +405,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="18.71" bestFit="true" customWidth="true" style="0"/>
@@ -410,10 +416,12 @@
     <col min="6" max="6" width="26.993" bestFit="true" customWidth="true" style="0"/>
     <col min="7" max="7" width="13.997" bestFit="true" customWidth="true" style="0"/>
     <col min="8" max="8" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="9" max="9" width="34.135" bestFit="true" customWidth="true" style="0"/>
+    <col min="9" max="9" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="10" max="10" width="34.135" bestFit="true" customWidth="true" style="0"/>
+    <col min="11" max="11" width="34.135" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,25 +449,31 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G2">
         <v>25</v>
@@ -468,7 +482,13 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>50</v>
+        <v>10</v>
+      </c>
+      <c r="J2">
+        <v>15</v>
+      </c>
+      <c r="K2">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>